<commit_message>
Edits to do with making folders relative and data synthetic, probably
</commit_message>
<xml_diff>
--- a/0. Example exported from overview code.xlsx
+++ b/0. Example exported from overview code.xlsx
@@ -69,7 +69,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">1,657</t>
+    <t xml:space="preserve">1,638</t>
   </si>
   <si>
     <t xml:space="preserve">Sex of respondent
@@ -628,13 +628,13 @@
         <v>15</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>84.9</v>
+        <v>85</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>84.3</v>
+        <v>87</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>85.4</v>
+        <v>83.5</v>
       </c>
     </row>
     <row r="6">
@@ -645,13 +645,13 @@
         <v>15</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>4.7</v>
+        <v>5.1</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>4.6</v>
+        <v>3.7</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>4.8</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="7">
@@ -662,13 +662,13 @@
         <v>15</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="8">
@@ -679,13 +679,13 @@
         <v>15</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>3.2</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="9">
@@ -696,13 +696,13 @@
         <v>15</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>1.8</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="10">
@@ -713,13 +713,13 @@
         <v>15</v>
       </c>
       <c r="D10" s="11" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="E10" s="11" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>2.1</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="11">
@@ -730,13 +730,13 @@
         <v>15</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="12">
@@ -784,10 +784,10 @@
         <v>17</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>759</v>
+        <v>737</v>
       </c>
       <c r="F14" s="18" t="n">
-        <v>898</v>
+        <v>901</v>
       </c>
     </row>
     <row r="15">

</xml_diff>